<commit_message>
Added extra footnotes following 2025 publication
</commit_message>
<xml_diff>
--- a/reference-files/qom-template.xlsx
+++ b/reference-files/qom-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\irf\18-End-of-Life\Publication\Sissi\end-of-life-pub\reference-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC74F8B3-F913-44F1-81AB-F187C15981AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193B40C2-D50C-44D8-837A-76FD39CC9C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="888" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="888" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="232">
   <si>
     <t>Borders</t>
   </si>
@@ -475,9 +475,6 @@
     <t>Clackmannanshire and Stirling</t>
   </si>
   <si>
-    <t>These statistics are derived from data collected on discharges from acute and community hospitals (SMR01), pyschiatric hospitals (SMR04) and geriatric long stay facilities (SMR01 GLS) in Scotland.</t>
-  </si>
-  <si>
     <t>4.</t>
   </si>
   <si>
@@ -841,6 +838,15 @@
   <si>
     <t>https://www.gov.scot/publications/scottish-government-urban-rural-classification-2022</t>
   </si>
+  <si>
+    <t>These statistics are derived from data collected on discharges from acute and community hospitals (SMR01), pyschiatric hospitals (SMR04) and geriatric long stay facilities (SMR01 GLS) in Scotland. Figures for the last year are provisional.</t>
+  </si>
+  <si>
+    <t>Provisional note for latest f. year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See data completeness tables in Appendix 2 of report. </t>
+  </si>
 </sst>
 </file>
 
@@ -851,7 +857,7 @@
     <numFmt numFmtId="165" formatCode="#.00"/>
     <numFmt numFmtId="166" formatCode="#.0"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1020,6 +1026,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1117,7 +1130,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1351,6 +1364,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="14" applyFont="1"/>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2963,8 +2981,27 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>= % of time at home or in a community 				               setting in last 6 months of life x 182.5</a:t>
+            <a:t>= (% of time at home or in a community 				                                                                   setting in last 6 months of life x 182.5) / 100</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr sz="1000"/>
+          </a:pPr>
           <a:endParaRPr lang="en-GB" sz="1200">
             <a:effectLst/>
             <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
@@ -3758,7 +3795,8 @@
   <cols>
     <col min="1" max="1" width="1.6640625" style="33" customWidth="1"/>
     <col min="2" max="2" width="3.44140625" style="33" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="33"/>
+    <col min="3" max="13" width="11.5546875" style="33" customWidth="1"/>
+    <col min="14" max="16384" width="9.109375" style="33"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3787,7 +3825,7 @@
     </row>
     <row r="4" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3809,27 +3847,27 @@
     </row>
     <row r="6" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="37" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O6" s="37"/>
       <c r="P6" s="36"/>
     </row>
     <row r="7" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O7" s="37"/>
       <c r="P7" s="36"/>
     </row>
     <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="37" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P8" s="36"/>
     </row>
     <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C9" s="37"/>
       <c r="D9" s="37"/>
@@ -3848,7 +3886,7 @@
     </row>
     <row r="10" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="37" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
@@ -3867,7 +3905,7 @@
     </row>
     <row r="11" spans="2:16" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="38" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C11" s="33"/>
       <c r="D11" s="33"/>
@@ -3903,7 +3941,7 @@
     </row>
     <row r="13" spans="2:16" s="39" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="97" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C13" s="97"/>
       <c r="D13" s="97"/>
@@ -3922,7 +3960,7 @@
     </row>
     <row r="14" spans="2:16" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="82" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C14" s="33"/>
       <c r="D14" s="33"/>
@@ -3949,7 +3987,7 @@
     </row>
     <row r="18" spans="2:16" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C18" s="94" t="e">
         <f ca="1" xml:space="preserve"> calculation!$E$15</f>
@@ -3972,7 +4010,7 @@
     <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13"/>
       <c r="C19" s="96" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D19" s="96"/>
       <c r="E19" s="96"/>
@@ -4009,7 +4047,7 @@
         <v>13</v>
       </c>
       <c r="C21" s="97" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D21" s="97"/>
       <c r="E21" s="97"/>
@@ -4046,7 +4084,7 @@
         <v>85</v>
       </c>
       <c r="C23" s="94" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D23" s="95"/>
       <c r="E23" s="95"/>
@@ -4387,7 +4425,7 @@
     </row>
     <row r="43" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C43" s="42" t="s">
         <v>86</v>
@@ -4408,10 +4446,10 @@
     </row>
     <row r="45" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="46" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4431,7 +4469,7 @@
     <row r="47" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="15"/>
       <c r="C47" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D47" s="17"/>
       <c r="E47" s="16"/>
@@ -4452,7 +4490,7 @@
         <v>109</v>
       </c>
       <c r="C49" s="95" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D49" s="95"/>
       <c r="E49" s="95"/>
@@ -4475,10 +4513,10 @@
     <row r="51" spans="1:16" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="13"/>
       <c r="B51" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C51" s="94" t="s">
-        <v>133</v>
+        <v>229</v>
       </c>
       <c r="D51" s="95"/>
       <c r="E51" s="95"/>
@@ -4497,6 +4535,9 @@
     <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="13"/>
       <c r="B52" s="13"/>
+      <c r="C52" s="104" t="s">
+        <v>139</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -4523,11 +4564,12 @@
     <hyperlink ref="B11" location="'Table 6 - LA'!A1" display="Table 6: Percentage of time in the last six months of life spent at home or in a community setting; by Local Authority" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="C19" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="C19:P19" r:id="rId2" display="See Appendix 2 of the full report for more information." xr:uid="{9A743234-A722-4414-A174-CB6A57800D63}"/>
+    <hyperlink ref="C52" r:id="rId3" xr:uid="{79B22F25-4A74-4786-87B4-2593234D930E}"/>
   </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="70" orientation="landscape" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="70" orientation="landscape" r:id="rId4"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -4543,12 +4585,12 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="86" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="B3" s="86" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -4646,7 +4688,7 @@
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
@@ -4659,12 +4701,12 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
@@ -4681,7 +4723,7 @@
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -4694,7 +4736,7 @@
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
@@ -4713,7 +4755,7 @@
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="89" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
@@ -4789,14 +4831,14 @@
     </row>
     <row r="2" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="85" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J2" s="64"/>
       <c r="K2" s="64"/>
     </row>
     <row r="3" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J3" s="64"/>
       <c r="K3" s="64"/>
@@ -4809,7 +4851,7 @@
     <row r="5" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="J5" s="64"/>
       <c r="L5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4825,7 +4867,7 @@
     </row>
     <row r="7" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="24" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C7" s="4" t="e">
         <f ca="1">calculation!B$10</f>
@@ -5005,7 +5047,7 @@
     </row>
     <row r="11" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C11" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B11), [0]!data_range, 5, FALSE)</f>
@@ -5050,7 +5092,7 @@
     </row>
     <row r="12" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="64" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C12" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B12), [0]!data_range, 5, FALSE)</f>
@@ -5095,7 +5137,7 @@
     </row>
     <row r="13" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C13" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B13), [0]!data_range, 5, FALSE)</f>
@@ -5140,7 +5182,7 @@
     </row>
     <row r="14" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="64" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C14" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B14), [0]!data_range, 5, FALSE)</f>
@@ -5185,7 +5227,7 @@
     </row>
     <row r="15" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="64" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C15" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B15), [0]!data_range, 5, FALSE)</f>
@@ -5905,7 +5947,7 @@
     </row>
     <row r="31" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="64" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C31" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B31), [0]!data_range, 5, FALSE)</f>
@@ -6175,7 +6217,7 @@
     </row>
     <row r="37" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="64" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C37" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "ca", $B37), [0]!data_range, 5, FALSE)</f>
@@ -6371,14 +6413,14 @@
     </row>
     <row r="44" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J44" s="64"/>
       <c r="K44" s="64"/>
     </row>
     <row r="45" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J45" s="64"/>
       <c r="K45" s="64"/>
@@ -7712,7 +7754,7 @@
     <row r="44" spans="1:3" s="58" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="77"/>
       <c r="B44" s="62" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="58" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7727,7 +7769,7 @@
     <row r="47" spans="1:3" s="58" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="77"/>
       <c r="B47" s="78" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C47" s="79"/>
     </row>
@@ -8111,19 +8153,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" t="s">
         <v>145</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>146</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>147</v>
-      </c>
-      <c r="E1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -27047,7 +27089,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B1">
         <f>COUNTA(data!B:B)-1</f>
@@ -27056,7 +27098,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B2">
         <f>COUNTA(data!1:1)</f>
@@ -27065,26 +27107,26 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="81" t="s">
         <v>188</v>
-      </c>
-      <c r="B5" s="81" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="83" t="s">
         <v>186</v>
-      </c>
-      <c r="B6" s="83" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -27184,13 +27226,13 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D13" t="s">
+        <v>180</v>
+      </c>
+      <c r="E13" t="s">
         <v>181</v>
-      </c>
-      <c r="E13" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -27201,7 +27243,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E14" t="e">
         <f ca="1">"Data for "&amp; $K$9 &amp;" are provisional. Please see Notes tab for more information."</f>
@@ -27213,10 +27255,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E15" s="103" t="e">
         <f ca="1">IF($E$13 = "provisional", "Hospital data and ", "") &amp; "National Records of Scotland deaths data " &amp; IF($E$13 = "provisional", "are", "is") &amp; " provisional for " &amp; $K$9 &amp;". " &amp; IF($E$13 = "provisional", "This publication will be updated in October 20" &amp; RIGHT($K$9,2) &amp; ". " &amp; $E$16, "")</f>
@@ -27237,10 +27279,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -27251,7 +27293,7 @@
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E17" s="1" t="str">
         <f>"Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays."</f>
@@ -27271,7 +27313,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -27281,6 +27323,13 @@
       <c r="B20" t="s">
         <v>4</v>
       </c>
+      <c r="D20" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="E20" t="e">
+        <f ca="1">"Data for "&amp; $K$9 &amp;" are provisional. Please see Notes tab for more information. Where hospital completeness is lower, this may impact the amount of time spent at home or in the community."</f>
+        <v>#REF!</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
@@ -27367,7 +27416,7 @@
         <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -27383,7 +27432,7 @@
         <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -27431,7 +27480,7 @@
         <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -27519,7 +27568,7 @@
         <v>24</v>
       </c>
       <c r="B51" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -27591,7 +27640,7 @@
         <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -27599,7 +27648,7 @@
         <v>2</v>
       </c>
       <c r="B62" s="32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -27607,7 +27656,7 @@
         <v>3</v>
       </c>
       <c r="B63" s="32" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -27615,7 +27664,7 @@
         <v>4</v>
       </c>
       <c r="B64" s="32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -27623,7 +27672,7 @@
         <v>5</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -27631,7 +27680,7 @@
         <v>1</v>
       </c>
       <c r="B67" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -27639,7 +27688,7 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -27647,7 +27696,7 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -27655,7 +27704,7 @@
         <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -27663,7 +27712,7 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -27671,7 +27720,7 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -27690,7 +27739,7 @@
   <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:M65"/>
+  <dimension ref="B1:M66"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.6640625" style="1" customWidth="1"/>
@@ -27724,7 +27773,7 @@
     </row>
     <row r="3" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I3" s="64"/>
       <c r="J3" s="64"/>
@@ -27741,7 +27790,7 @@
       <c r="J5" s="64"/>
       <c r="K5" s="19"/>
       <c r="L5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -27757,7 +27806,7 @@
     </row>
     <row r="7" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C7" s="4" t="e">
         <f ca="1">calculation!B$10</f>
@@ -27803,7 +27852,7 @@
     </row>
     <row r="8" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="65" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C8" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hb", "NHS ", $B8), [0]!data_range, 5, FALSE)</f>
@@ -27895,7 +27944,7 @@
     </row>
     <row r="10" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C10" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hb", "NHS ", $B10), [0]!data_range, 5, FALSE)</f>
@@ -28079,7 +28128,7 @@
     </row>
     <row r="14" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C14" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hb", "NHS ", $B14), [0]!data_range, 5, FALSE)</f>
@@ -28506,7 +28555,7 @@
     </row>
     <row r="26" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -28517,7 +28566,7 @@
     </row>
     <row r="27" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -28528,7 +28577,7 @@
     </row>
     <row r="28" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$20</f>
         <v>#REF!</v>
       </c>
       <c r="E28" s="6"/>
@@ -28539,9 +28588,8 @@
       <c r="K28" s="64"/>
     </row>
     <row r="29" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="5" t="str">
-        <f>"1. " &amp; calculation!E17</f>
-        <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
+      <c r="B29" s="89" t="s">
+        <v>231</v>
       </c>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
@@ -28551,6 +28599,10 @@
       <c r="K29" s="64"/>
     </row>
     <row r="30" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="str">
+        <f>"1. " &amp; calculation!E17</f>
+        <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
+      </c>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
@@ -28623,6 +28675,9 @@
       <c r="K38" s="64"/>
     </row>
     <row r="39" spans="5:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
       <c r="I39" s="64"/>
       <c r="J39" s="64"/>
       <c r="K39" s="64"/>
@@ -28756,6 +28811,11 @@
       <c r="I65" s="64"/>
       <c r="J65" s="64"/>
       <c r="K65" s="64"/>
+    </row>
+    <row r="66" spans="9:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I66" s="64"/>
+      <c r="J66" s="64"/>
+      <c r="K66" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -28764,9 +28824,10 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B24" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B29" r:id="rId1" xr:uid="{7A8FE3B8-5D01-4A4E-AAC7-0FFC95EB58AB}"/>
   </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="93" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="93" orientation="landscape" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
@@ -28774,7 +28835,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A2:W38"/>
+  <dimension ref="A2:W39"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.6640625" style="1" customWidth="1"/>
@@ -28783,7 +28844,7 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="86" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -28887,7 +28948,7 @@
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -28900,22 +28961,27 @@
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="30" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$20</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="5" t="str">
+      <c r="B38" s="105" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="5" t="str">
         <f>"1. " &amp; calculation!E17</f>
         <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
       </c>
@@ -28923,17 +28989,18 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B33" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="B38" r:id="rId1" xr:uid="{FA7DA054-232B-4146-841B-8A10E14AAF32}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
+  <legacyDrawing r:id="rId4"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="3074" r:id="rId4" name="Drop Down 2">
+            <control shapeId="3074" r:id="rId5" name="Drop Down 2">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -28997,7 +29064,7 @@
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J3" s="64"/>
       <c r="K3" s="64"/>
@@ -29013,7 +29080,7 @@
       <c r="J5" s="64"/>
       <c r="K5" s="19"/>
       <c r="L5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29274,7 +29341,7 @@
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C11" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hscp", $B11), [0]!data_range, 5, FALSE)</f>
@@ -29402,7 +29469,7 @@
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="64" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C13" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hscp", $B13), [0]!data_range, 5, FALSE)</f>
@@ -29786,7 +29853,7 @@
     </row>
     <row r="19" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="64" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C19" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hscp", $B19), [0]!data_range, 5, FALSE)</f>
@@ -30490,7 +30557,7 @@
     </row>
     <row r="30" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="64" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C30" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "hscp", $B30), [0]!data_range, 5, FALSE)</f>
@@ -31154,7 +31221,7 @@
     </row>
     <row r="44" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J44" s="64"/>
       <c r="K44" s="64"/>
@@ -31162,7 +31229,7 @@
     </row>
     <row r="45" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J45" s="64"/>
       <c r="K45" s="64"/>
@@ -31170,7 +31237,7 @@
     </row>
     <row r="46" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="30" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$20</f>
         <v>#REF!</v>
       </c>
       <c r="J46" s="64"/>
@@ -31178,15 +31245,18 @@
       <c r="L46" s="67"/>
     </row>
     <row r="47" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="5" t="str">
-        <f>"1. " &amp; calculation!E17</f>
-        <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
+      <c r="B47" s="105" t="s">
+        <v>231</v>
       </c>
       <c r="J47" s="64"/>
       <c r="K47" s="64"/>
       <c r="L47" s="67"/>
     </row>
     <row r="48" spans="2:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="5" t="str">
+        <f>"1. " &amp; calculation!E17</f>
+        <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
+      </c>
       <c r="J48" s="64"/>
       <c r="K48" s="64"/>
       <c r="L48" s="67"/>
@@ -31896,9 +31966,10 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B42" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="B47" r:id="rId1" xr:uid="{F9CF39AA-359C-4606-8E6C-E3DA0590E2C1}"/>
   </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="63" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="63" orientation="portrait" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
@@ -31906,7 +31977,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A2:W38"/>
+  <dimension ref="A2:W39"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.6640625" style="1" customWidth="1"/>
@@ -31915,7 +31986,7 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="86" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
@@ -32019,7 +32090,7 @@
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -32032,22 +32103,27 @@
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="30" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$E$20</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="5" t="str">
+      <c r="B38" s="106" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="5" t="str">
         <f>"1. " &amp; calculation!E17</f>
         <v>1. Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays.</v>
       </c>
@@ -32055,16 +32131,17 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B33" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="B38" r:id="rId1" xr:uid="{5F307BC7-3F16-438F-9735-C03AE4C48A2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="7169" r:id="rId3" name="Drop Down 1">
+            <control shapeId="7169" r:id="rId4" name="Drop Down 1">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -32129,7 +32206,7 @@
     </row>
     <row r="3" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J3" s="64"/>
       <c r="K3" s="64"/>
@@ -32148,7 +32225,7 @@
       <c r="K5" s="64"/>
       <c r="L5" s="64"/>
       <c r="M5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -32168,7 +32245,7 @@
         <v>117</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D7" s="4" t="e">
         <f ca="1">calculation!B$10</f>
@@ -32213,7 +32290,7 @@
     </row>
     <row r="8" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>112</v>
@@ -32261,7 +32338,7 @@
     </row>
     <row r="9" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D9" s="90" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$8, " ", $C9), [0]!data_range, 5, FALSE)</f>
@@ -32351,7 +32428,7 @@
     </row>
     <row r="11" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>112</v>
@@ -32399,7 +32476,7 @@
     </row>
     <row r="12" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D12" s="90" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$11, " ", $C12), [0]!data_range, 5, FALSE)</f>
@@ -32489,7 +32566,7 @@
     </row>
     <row r="14" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>112</v>
@@ -32537,7 +32614,7 @@
     </row>
     <row r="15" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D15" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$14, " ", $C15), [0]!data_range, 5, FALSE)</f>
@@ -32675,7 +32752,7 @@
     </row>
     <row r="18" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D18" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$17, " ", $C18), [0]!data_range, 5, FALSE)</f>
@@ -32813,7 +32890,7 @@
     </row>
     <row r="21" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D21" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$20, " ", $C21), [0]!data_range, 5, FALSE)</f>
@@ -32951,7 +33028,7 @@
     </row>
     <row r="24" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D24" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$23, " ", $C24), [0]!data_range, 5, FALSE)</f>
@@ -33089,7 +33166,7 @@
     </row>
     <row r="27" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D27" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$26, " ", $C27), [0]!data_range, 5, FALSE)</f>
@@ -33227,7 +33304,7 @@
     </row>
     <row r="30" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D30" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(D$7, 7), "age/sex", $B$29, " ", $C30), [0]!data_range, 5, FALSE)</f>
@@ -33337,7 +33414,7 @@
     </row>
     <row r="35" spans="2:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="99" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C35" s="99"/>
       <c r="D35" s="99"/>
@@ -33363,12 +33440,12 @@
     </row>
     <row r="37" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="38" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33493,13 +33570,13 @@
     </row>
     <row r="2" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="85" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L2" s="69"/>
     </row>
     <row r="3" spans="2:18" ht="18" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I3" s="64"/>
       <c r="J3" s="64"/>
@@ -33519,7 +33596,7 @@
       <c r="J5" s="64"/>
       <c r="K5" s="64"/>
       <c r="L5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33535,7 +33612,7 @@
     </row>
     <row r="7" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="24" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C7" s="4" t="e">
         <f ca="1">calculation!B$10</f>
@@ -33586,7 +33663,7 @@
     </row>
     <row r="8" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "simd quintile", $B8), [0]!data_range, 5, FALSE)</f>
@@ -33790,7 +33867,7 @@
     </row>
     <row r="12" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="29" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C12" s="8" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "simd quintile", $B12), [0]!data_range, 5, FALSE)</f>
@@ -33877,7 +33954,7 @@
     </row>
     <row r="15" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C15" s="4" t="e">
         <f ca="1">calculation!B$10</f>
@@ -34056,12 +34133,12 @@
     </row>
     <row r="22" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="2:18" s="45" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34078,7 +34155,7 @@
     </row>
     <row r="26" spans="2:18" s="45" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="99" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C26" s="99"/>
       <c r="D26" s="99"/>
@@ -34102,7 +34179,7 @@
     </row>
     <row r="28" spans="2:18" s="45" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C28" s="72"/>
       <c r="D28" s="73"/>
@@ -34211,12 +34288,12 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="86" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.3">
       <c r="B3" s="86" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -34314,7 +34391,7 @@
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
@@ -34327,7 +34404,7 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F35" s="30"/>
       <c r="G35" s="30"/>
@@ -34337,7 +34414,7 @@
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
@@ -34370,7 +34447,7 @@
     </row>
     <row r="39" spans="2:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="100" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C39" s="100"/>
       <c r="D39" s="100"/>
@@ -34467,7 +34544,7 @@
     </row>
     <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L2" s="67"/>
       <c r="M2" s="69"/>
@@ -34475,7 +34552,7 @@
     </row>
     <row r="3" spans="2:19" ht="18" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L3" s="67"/>
       <c r="M3" s="69"/>
@@ -34488,7 +34565,7 @@
     </row>
     <row r="5" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L5" s="52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="M5" s="69"/>
       <c r="N5" s="69"/>
@@ -34561,7 +34638,7 @@
     </row>
     <row r="8" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C8" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B8), [0]!data_range, 5, FALSE)</f>
@@ -34613,7 +34690,7 @@
     </row>
     <row r="9" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B9), [0]!data_range, 5, FALSE)</f>
@@ -34665,7 +34742,7 @@
     </row>
     <row r="10" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C10" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B10), [0]!data_range, 5, FALSE)</f>
@@ -34717,7 +34794,7 @@
     </row>
     <row r="11" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C11" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B11), [0]!data_range, 5, FALSE)</f>
@@ -34769,7 +34846,7 @@
     </row>
     <row r="12" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C12" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B12), [0]!data_range, 5, FALSE)</f>
@@ -34821,7 +34898,7 @@
     </row>
     <row r="13" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C13" s="8" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$7, 7), "urban rural 6", $B13), [0]!data_range, 5, FALSE)</f>
@@ -34943,7 +35020,7 @@
     </row>
     <row r="17" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C17" s="6" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$16, 7), "urban rural 2", $B17), [0]!data_range, 5, FALSE)</f>
@@ -34995,7 +35072,7 @@
     </row>
     <row r="18" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C18" s="8" t="e">
         <f ca="1">VLOOKUP(CONCATENATE(LEFT(C$16, 7), "urban rural 2", $B18), [0]!data_range, 5, FALSE)</f>
@@ -35064,7 +35141,7 @@
     </row>
     <row r="22" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L22" s="67"/>
       <c r="M22" s="69"/>
@@ -35072,7 +35149,7 @@
     </row>
     <row r="23" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L23" s="67"/>
       <c r="M23" s="69"/>
@@ -35102,7 +35179,7 @@
     </row>
     <row r="26" spans="2:19" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -35115,7 +35192,7 @@
     </row>
     <row r="27" spans="2:19" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -35132,7 +35209,7 @@
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="89" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>

</xml_diff>